<commit_message>
sign fix for basis
</commit_message>
<xml_diff>
--- a/PROJECT-CTD-FINANCING-WS.xlsx
+++ b/PROJECT-CTD-FINANCING-WS.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Nikolas\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3E437DC0-3EF6-465A-A1BD-90162A513E92}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D60B9668-247D-4EFC-B66B-B9266A4075D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3DCF5A8D-45A8-43FD-93EA-9C8C9B9C0CC5}"/>
   </bookViews>
@@ -858,12 +858,12 @@
         <v>99.562314358974348</v>
       </c>
       <c r="X5" s="4">
-        <f>V5-P5</f>
-        <v>0.39363304029303947</v>
+        <f>P5-V5</f>
+        <v>-0.39363304029303947</v>
       </c>
       <c r="Y5" s="9">
-        <f>W5-P5</f>
-        <v>1.3057209523809519</v>
+        <f>P5-W5</f>
+        <v>-1.3057209523809519</v>
       </c>
       <c r="Z5" s="4"/>
       <c r="AA5" s="4">
@@ -879,12 +879,12 @@
         <v>90.841087912087914</v>
       </c>
       <c r="AD5" s="4">
-        <f>AB5-P5</f>
-        <v>-8.3275934065933939</v>
+        <f>P5-AB5</f>
+        <v>8.3275934065933939</v>
       </c>
       <c r="AE5" s="9">
-        <f>AC5-P5</f>
-        <v>-7.4155054945054815</v>
+        <f>P5-AC5</f>
+        <v>7.4155054945054815</v>
       </c>
     </row>
     <row r="6" spans="1:31" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -957,12 +957,12 @@
         <v>100.34735002747253</v>
       </c>
       <c r="X6" s="5">
-        <f>V6-P6</f>
-        <v>5.2844532967029068E-2</v>
+        <f>P6-V6</f>
+        <v>-5.2844532967029068E-2</v>
       </c>
       <c r="Y6" s="10">
-        <f>W6-P6</f>
-        <v>1.2410313461538465</v>
+        <f>P6-W6</f>
+        <v>-1.2410313461538465</v>
       </c>
       <c r="Z6" s="5"/>
       <c r="AA6" s="5">
@@ -978,12 +978,12 @@
         <v>94.384311813186827</v>
       </c>
       <c r="AD6" s="5">
-        <f>AB6-P6</f>
-        <v>-5.910193681318674</v>
+        <f>P6-AB6</f>
+        <v>5.910193681318674</v>
       </c>
       <c r="AE6" s="10">
-        <f>AC6-P6</f>
-        <v>-4.7220068681318565</v>
+        <f>P6-AC6</f>
+        <v>4.7220068681318565</v>
       </c>
     </row>
     <row r="7" spans="1:31" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -1056,12 +1056,12 @@
         <v>100.06475010683761</v>
       </c>
       <c r="X7" s="4">
-        <f t="shared" ref="X7:X29" si="8">V7-P7</f>
-        <v>-0.83195318986568623</v>
+        <f t="shared" ref="X7:X29" si="8">P7-V7</f>
+        <v>0.83195318986568623</v>
       </c>
       <c r="Y7" s="9">
-        <f t="shared" ref="Y7:Y29" si="9">W7-P7</f>
-        <v>0.44551933760683937</v>
+        <f t="shared" ref="Y7:Y29" si="9">P7-W7</f>
+        <v>-0.44551933760683937</v>
       </c>
       <c r="Z7" s="4"/>
       <c r="AA7" s="4">
@@ -1077,12 +1077,12 @@
         <v>97.408472527472526</v>
       </c>
       <c r="AD7" s="4">
-        <f t="shared" ref="AD7:AD29" si="12">AB7-P7</f>
-        <v>-3.4882307692307677</v>
+        <f t="shared" ref="AD7:AD29" si="12">P7-AB7</f>
+        <v>3.4882307692307677</v>
       </c>
       <c r="AE7" s="9">
-        <f t="shared" ref="AE7:AE29" si="13">AC7-P7</f>
-        <v>-2.2107582417582421</v>
+        <f t="shared" ref="AE7:AE29" si="13">P7-AC7</f>
+        <v>2.2107582417582421</v>
       </c>
     </row>
     <row r="8" spans="1:31" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -1156,11 +1156,11 @@
       </c>
       <c r="X8" s="5">
         <f t="shared" si="8"/>
-        <v>-0.55535679487179834</v>
+        <v>0.55535679487179834</v>
       </c>
       <c r="Y8" s="10">
         <f t="shared" si="9"/>
-        <v>1.1850278205128149</v>
+        <v>-1.1850278205128149</v>
       </c>
       <c r="Z8" s="5"/>
       <c r="AA8" s="5">
@@ -1177,11 +1177,11 @@
       </c>
       <c r="AD8" s="5">
         <f t="shared" si="12"/>
-        <v>-1.463019230769234</v>
+        <v>1.463019230769234</v>
       </c>
       <c r="AE8" s="10">
         <f t="shared" si="13"/>
-        <v>0.27736538461537918</v>
+        <v>-0.27736538461537918</v>
       </c>
     </row>
     <row r="9" spans="1:31" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -1255,11 +1255,11 @@
       </c>
       <c r="X9" s="4">
         <f t="shared" si="8"/>
-        <v>-0.64843343101343009</v>
+        <v>0.64843343101343009</v>
       </c>
       <c r="Y9" s="9">
         <f t="shared" si="9"/>
-        <v>1.1427753601953583</v>
+        <v>-1.1427753601953583</v>
       </c>
       <c r="Z9" s="4"/>
       <c r="AA9" s="4">
@@ -1276,11 +1276,11 @@
       </c>
       <c r="AD9" s="4">
         <f t="shared" si="12"/>
-        <v>0.70278021978022309</v>
+        <v>-0.70278021978022309</v>
       </c>
       <c r="AE9" s="9">
         <f t="shared" si="13"/>
-        <v>2.4939890109890115</v>
+        <v>-2.4939890109890115</v>
       </c>
     </row>
     <row r="10" spans="1:31" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -1354,11 +1354,11 @@
       </c>
       <c r="X10" s="5">
         <f t="shared" si="8"/>
-        <v>-1.1923101266788763</v>
+        <v>1.1923101266788763</v>
       </c>
       <c r="Y10" s="10">
         <f t="shared" si="9"/>
-        <v>1.1195030601343063</v>
+        <v>-1.1195030601343063</v>
       </c>
       <c r="Z10" s="5"/>
       <c r="AA10" s="5">
@@ -1375,11 +1375,11 @@
       </c>
       <c r="AD10" s="5">
         <f t="shared" si="12"/>
-        <v>2.6917994505494391</v>
+        <v>-2.6917994505494391</v>
       </c>
       <c r="AE10" s="10">
         <f t="shared" si="13"/>
-        <v>5.0036126373626217</v>
+        <v>-5.0036126373626217</v>
       </c>
     </row>
     <row r="11" spans="1:31" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -1453,11 +1453,11 @@
       </c>
       <c r="X11" s="4">
         <f t="shared" si="8"/>
-        <v>-1.0941640354090225</v>
+        <v>1.0941640354090225</v>
       </c>
       <c r="Y11" s="9">
         <f t="shared" si="9"/>
-        <v>1.0899018986569047</v>
+        <v>-1.0899018986569047</v>
       </c>
       <c r="Z11" s="4"/>
       <c r="AA11" s="4">
@@ -1474,11 +1474,11 @@
       </c>
       <c r="AD11" s="4">
         <f t="shared" si="12"/>
-        <v>5.5114203296703437</v>
+        <v>-5.5114203296703437</v>
       </c>
       <c r="AE11" s="9">
         <f t="shared" si="13"/>
-        <v>7.6954862637362851</v>
+        <v>-7.6954862637362851</v>
       </c>
     </row>
     <row r="12" spans="1:31" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -2936,15 +2936,15 @@
       </c>
       <c r="G33" s="4">
         <f>_xlfn.AGGREGATE(15,6,AE5:AE29,1)</f>
-        <v>-7.4155054945054815</v>
+        <v>-7.6954862637362851</v>
       </c>
       <c r="H33" s="4">
         <f>_xlfn.AGGREGATE(15,6,Y5:Y29,1)</f>
-        <v>0.44551933760683937</v>
+        <v>-1.3057209523809519</v>
       </c>
       <c r="I33" s="4">
         <f>G33-H33</f>
-        <v>-7.8610248321123208</v>
+        <v>-6.3897653113553332</v>
       </c>
       <c r="J33" s="4" t="str">
         <f>IF(I33&gt;0,"Rich",IF(I33&lt;0,"Cheap","Fair"))</f>

</xml_diff>